<commit_message>
add solder bumper instead of pull-up at EEPROM write access protection pin; generate production files
</commit_message>
<xml_diff>
--- a/Project Outputs for UZ_D_Resolver/Rev02/BOM/BOM_JLC-UZ_D_Resolver(Default).xlsx
+++ b/Project Outputs for UZ_D_Resolver/Rev02/BOM/BOM_JLC-UZ_D_Resolver(Default).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projekte\UltraZohm\Work_Altium\uz_d_resolver\Project Outputs for UZ_D_Resolver\Rev02\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BCFD77C2-96D7-49D1-9014-58A885825E7C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4BCE0C49-0953-4483-ADA8-5BDA49B81362}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="10215" xr2:uid="{7B1CB551-F52E-49A9-BFCD-BA492A3F477C}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="10215" xr2:uid="{1273805D-D129-48DF-AC43-A740BE1818E3}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC-UZ_D_Resolver(Default)" sheetId="1" r:id="rId1"/>
@@ -372,7 +372,7 @@
     <t>4k7</t>
   </si>
   <si>
-    <t>R22A, R22B, R22C, R46A, R46B, R46C, R47A, R47B, R47C, R48A, R48B, R48C, R49A, R49B, R49C, R56, R57</t>
+    <t>R22A, R22B, R22C, R46A, R46B, R46C, R47A, R47B, R47C, R48A, R48B, R48C, R49A, R49B, R49C, R55, R56, R57</t>
   </si>
   <si>
     <t>UNI-ROYAL</t>
@@ -946,7 +946,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1849F93E-621C-41AA-8211-EF0089BC7336}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A395C4F-DE04-45F3-88BC-41BA9CF9E93B}">
   <dimension ref="A1:K35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1556,7 +1556,7 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>113</v>

</xml_diff>